<commit_message>
Add initial V3 robot sorting program
Add new robot control script code/src/v3.py for the White-Stripes IQ2 project. The script configures motors, sensors (distance, optical, AI vision), and LEDs; implements two sorting modes (color and AprilTag), pickup/drop routines, UI helpers, and counters for sorted boxes. Includes LED/state notes and main loop to drive, detect, pick, and place objects. Also add White-Stripes Code Notes.xlsx containing project documentation/notes.
</commit_message>
<xml_diff>
--- a/White-Stripes Code Notes.xlsx
+++ b/White-Stripes Code Notes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/62b4f05cfa1d15a8/Desktop/Ali Zain/Sunlake Academy 8th grade/Robotics 25-26/White-Stripes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="138" documentId="8_{5AC36F59-3A81-449C-AD00-DD8419A394EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97832A6D-40B3-45DD-96DA-77C8D730389F}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="8_{5AC36F59-3A81-449C-AD00-DD8419A394EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD3DE1D9-5461-493D-8999-5EA4A11D3DCF}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="7500" windowHeight="6000" xr2:uid="{B1289BB2-4135-4309-86E7-7A5724C50F26}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
   <si>
     <t>Notes</t>
   </si>
@@ -83,23 +83,38 @@
     <t>bugs (obsolete)</t>
   </si>
   <si>
-    <t>in development</t>
-  </si>
-  <si>
     <t>V2 + removed thread for sorting mode indicator, fixed sort by color green/blue problem, added comments, put main code in a special main() function, led now fades</t>
   </si>
   <si>
-    <t>V2.1 + lessened pick up height to prevent wheelies, fixed led fade problem on exit sorting indicator</t>
-  </si>
-  <si>
     <t>ground0</t>
+  </si>
+  <si>
+    <t>V2.1 + lessened pick up height to prevent wheelies</t>
+  </si>
+  <si>
+    <t>V2.2</t>
+  </si>
+  <si>
+    <t>V2.1 + controller input for hands free experience</t>
+  </si>
+  <si>
+    <t>ground0.1</t>
+  </si>
+  <si>
+    <t>V3</t>
+  </si>
+  <si>
+    <t>ground0 + V2.2</t>
+  </si>
+  <si>
+    <t>V2.1 + changed config for new robot design</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -109,6 +124,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -136,12 +159,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -159,9 +183,13 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1D8E4328-534B-470B-9C8F-4A7684F86A6D}" name="Table1" displayName="Table1" ref="A1:C7">
-  <autoFilter ref="A1:C7" xr:uid="{1D8E4328-534B-470B-9C8F-4A7684F86A6D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1D8E4328-534B-470B-9C8F-4A7684F86A6D}" name="Table1" displayName="Table1" ref="A1:C10">
+  <autoFilter ref="A1:C10" xr:uid="{1D8E4328-534B-470B-9C8F-4A7684F86A6D}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{1190CB18-7838-491C-B6C9-23F5C35AFA5C}" name="Version" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{E4A8B0BD-FD64-4843-BB76-31A9919809BC}" name="Notes"/>
@@ -488,7 +516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{646E6161-3125-44CA-BDAD-8EE4C165205A}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -556,21 +584,54 @@
         <v>13</v>
       </c>
       <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update robot main.py: wiring, sensors & sorting
Rework main robot program: remap motor and sensor ports, add a second LED, initialize sorting_mode and LED behavior, and set drivetrain velocities. Implement helper routines (brain_print, screen_prep), pickup/dropoff actions, color and AprilTag detection, box counters and display, and a working_lights thread to flash status LEDs. Add sorting flow for color and AprilTag modes with handling for multiple destinations and end sequence. Also add new empty v4.py and update White-Stripes Code Notes.xlsx (binary).
</commit_message>
<xml_diff>
--- a/White-Stripes Code Notes.xlsx
+++ b/White-Stripes Code Notes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/62b4f05cfa1d15a8/Desktop/Ali Zain/Sunlake Academy 8th grade/Robotics 25-26/White-Stripes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="164" documentId="8_{5AC36F59-3A81-449C-AD00-DD8419A394EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD3DE1D9-5461-493D-8999-5EA4A11D3DCF}"/>
+  <xr:revisionPtr revIDLastSave="175" documentId="8_{5AC36F59-3A81-449C-AD00-DD8419A394EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F821E76-F7F7-4670-AAC9-D4B8C03C7F13}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="7500" windowHeight="6000" xr2:uid="{B1289BB2-4135-4309-86E7-7A5724C50F26}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B1289BB2-4135-4309-86E7-7A5724C50F26}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
   <si>
     <t>Notes</t>
   </si>
@@ -83,6 +83,9 @@
     <t>bugs (obsolete)</t>
   </si>
   <si>
+    <t>in development</t>
+  </si>
+  <si>
     <t>V2 + removed thread for sorting mode indicator, fixed sort by color green/blue problem, added comments, put main code in a special main() function, led now fades</t>
   </si>
   <si>
@@ -108,6 +111,18 @@
   </si>
   <si>
     <t>V2.1 + changed config for new robot design</t>
+  </si>
+  <si>
+    <t>V4</t>
+  </si>
+  <si>
+    <t>V3 + new led funcionality (includes new added led), drift optimization, distance incorparation, box placing optimization</t>
+  </si>
+  <si>
+    <t>V4.1</t>
+  </si>
+  <si>
+    <t>V4 + one more led</t>
   </si>
 </sst>
 </file>
@@ -188,8 +203,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1D8E4328-534B-470B-9C8F-4A7684F86A6D}" name="Table1" displayName="Table1" ref="A1:C10">
-  <autoFilter ref="A1:C10" xr:uid="{1D8E4328-534B-470B-9C8F-4A7684F86A6D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1D8E4328-534B-470B-9C8F-4A7684F86A6D}" name="Table1" displayName="Table1" ref="A1:C12">
+  <autoFilter ref="A1:C12" xr:uid="{1D8E4328-534B-470B-9C8F-4A7684F86A6D}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{1190CB18-7838-491C-B6C9-23F5C35AFA5C}" name="Version" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{E4A8B0BD-FD64-4843-BB76-31A9919809BC}" name="Notes"/>
@@ -516,7 +531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{646E6161-3125-44CA-BDAD-8EE4C165205A}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -584,7 +599,7 @@
         <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
         <v>8</v>
@@ -592,10 +607,10 @@
     </row>
     <row r="7" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>8</v>
@@ -603,10 +618,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
         <v>8</v>
@@ -614,10 +629,10 @@
     </row>
     <row r="9" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>8</v>
@@ -625,13 +640,35 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>